<commit_message>
modified slt dictionary to fit the new stimuli of V1.2
</commit_message>
<xml_diff>
--- a/data_raw/SLT_dict.xlsx
+++ b/data_raw/SLT_dict.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anton\Nextcloud\Promotion\Tests\SLT\data_raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF55FA8A-8EF6-4811-B6B0-D7EDB91EA07B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F8D822A-3DAA-42D0-867A-13709147C462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="17115" windowHeight="10755" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="106">
   <si>
     <t>key</t>
   </si>
@@ -205,22 +205,6 @@
     <t>Nun geht es mit dem Haupttest los, in dem Ihre Ergebnisse gespeichert werden. \\ Ab jetzt bekommen Sie keine Rückmeldung mehr. Viel Erfolg!</t>
   </si>
   <si>
-    <t>Willkommen zum Melodie-Unterscheidungstest</t>
-  </si>
-  <si>
-    <t>Welcome to the Melody Discrimination Test</t>
-  </si>
-  <si>
-    <t>In dieser musikpsychologischen Studie möchten wir Deine musikalischen Hörfähigkeiten messen. Dafür haben wir einen Test entwickelt, in dem Du Melodien richtig erkennen und unterscheiden lernst.
-Ziel dieser Studie: Die Fähigkeit zu erfassen, Melodien zu erkennen und zu unterscheiden.
-Der Test dauert ca. 20 Minuten. Du solltest den Test in einem ruhigen Umfeld mit Kopfhörern oder einem guten Lautsprecher durchführen.</t>
-  </si>
-  <si>
-    <t>In dieser musikpsychologischen Studie möchten wir Ihre musikalischen Hörfähigkeiten messen. Dafür haben wir einen Test entwickelt, in dem Sie Melodien richtig erkennen und unterscheiden lernen.
-Ziel dieser Studie: Die Fähigkeit zu erfassen, Melodien zu erkennen und zu unterscheiden.
-Der Test dauert ca. 20 Minuten. Sie sollten den Test in einem ruhigen Umfeld mit Kopfhörern oder einem guten Lautsprecher durchführen.</t>
-  </si>
-  <si>
     <t>Du hast **{{accuracy}} %** der Melodien richtig erkannt.</t>
   </si>
   <si>
@@ -230,21 +214,6 @@
     <t>You recognized **{{accuracy}} %**  of the melodies correctly.</t>
   </si>
   <si>
-    <t>Du hast den Melodie-Unterscheidungstest erfolgreich beendet.</t>
-  </si>
-  <si>
-    <t>Sie haben den Melodie-Unterscheidungstest erfolgreich beendet.</t>
-  </si>
-  <si>
-    <t>You have completed the Melody Discrimination Test.</t>
-  </si>
-  <si>
-    <t>Melodie-Unterscheidungstest</t>
-  </si>
-  <si>
-    <t>Melody Discrimination Test</t>
-  </si>
-  <si>
     <t>Diese Melodie stammt von…</t>
   </si>
   <si>
@@ -263,112 +232,142 @@
     <t>FALSE_A</t>
   </si>
   <si>
-    <t>Du hörst gleich Melodien und sollst entscheiden, ob eine Melodie von Komponistin 1 oder von Komponistin 2 stammt. Das ist am Anfang noch sehr schwer, weil Du die Kompositionsstile der beiden nicht kennst und Du einfach raten musst.
-Aber keine Sorge, mit ein bisschen Übung kannst Du sicher alle Melodien gut zuordnen.</t>
-  </si>
-  <si>
-    <t>Sie hören gleich Melodien und sollen entscheiden, ob eine Melodie von Komponistin 1 oder von Komponistin 2 stammt. Das ist am Anfang noch sehr schwer, weil Sie die Kompositionsstile der beiden nicht kennen und einfach raten müssen.
-Aber keine Sorge, mit ein bisschen Übung können Sie sicher alle Melodien gut zuordnen.</t>
-  </si>
-  <si>
-    <t>You will soon hear melodies and should decide whether a melody was composed by Composer 1 or Composer 2.
-At the beginning this is quite difficult, because you don’t yet know their composing styles and will have to guess.
-But don’t worry — with a little practice you will surely be able to classify the melodies correctly.</t>
+    <t>Richtig, die Melodie stammt von Komponistin {{composer}}!</t>
+  </si>
+  <si>
+    <t>Richtig, die Melodie stammt von {{composer}}!</t>
+  </si>
+  <si>
+    <t>Falsch, die Melodie stammt von {{composer}}!</t>
+  </si>
+  <si>
+    <t>Correct, the melody was composed by {{composer}}!</t>
+  </si>
+  <si>
+    <t>False, the melody was composed by {{composer}}!</t>
+  </si>
+  <si>
+    <t>Falsch, die Melodie stammt von Komponistin {{composer}}!</t>
+  </si>
+  <si>
+    <t>FINAL_FEEDBACK_BLOCK1</t>
+  </si>
+  <si>
+    <t>FINAL_FEEDBACK_BLOCK2</t>
+  </si>
+  <si>
+    <t>FINAL_FEEDBACK_BLOCK3</t>
+  </si>
+  <si>
+    <t>Im ersten Block hast Du {{number_correct_1}} Melodien richtig zugeordnet.</t>
+  </si>
+  <si>
+    <t>Im ersten Block haben Sie {{number_correct_1}} Melodien richtig zugeordnet.</t>
+  </si>
+  <si>
+    <t>In the first block, you identified {{number_correct_1}} melodies correctly.</t>
+  </si>
+  <si>
+    <t>Im zweiten Block hast Du {{number_correct_2}} Melodien richtig zugeordnet.</t>
+  </si>
+  <si>
+    <t>Im zweiten Block haben Sie {{number_correct_2}} Melodien richtig zugeordnet.</t>
+  </si>
+  <si>
+    <t>In the second block, you identified {{number_correct_2}} melodies correctly.</t>
+  </si>
+  <si>
+    <t>Im dritten Block hast Du {{number_correct_3}} Melodien richtig zugeordnet.</t>
+  </si>
+  <si>
+    <t>Im dritten Block haben Sie {{number_correct_3}} Melodien richtig zugeordnet.</t>
+  </si>
+  <si>
+    <t>In the third block, you identified {{number_correct_3}} melodies correctly.</t>
+  </si>
+  <si>
+    <t>Welcome to the Statistical Learning Test</t>
+  </si>
+  <si>
+    <t>Willkommen zum Statistical Learning Test</t>
+  </si>
+  <si>
+    <t>In this test, we would like to measure your musical listening abilities. You will listen to short melodies and make judgements about what you hear.
+This task may feel difficult at first, especially at the beginning of the test. This is completely normal and expected. Please do not get discouraged if you are unsure about your answers, just go with your best guess and keep going.
+Please complete the test in a quiet environment using headphones or good-quality speakers.</t>
+  </si>
+  <si>
+    <t>In dieser Studie möchten wir deine  musikalische Hörfähigkeit messen. Du wirst kurze Melodien hören und beurteilen, was du hörst.
+Diese Aufgabe kann zunächst schwierig sein, besonders zu Beginn des Tests. Das ist völlig normal und zu erwarten. Bitte lass dich nicht entmutigen, wenn du bei deinen Antworten unsicher bist. Vertraue einfach auf deine beste Einschätzung.
+Bitte absolviere den Test in einer ruhigen Umgebung und verwende Kopfhörer oder Lautsprecher mit guter Klangqualität.</t>
+  </si>
+  <si>
+    <t>In dieser Studie möchten wir Ihre  musikalische Hörfähigkeit messen. Sie werden kurze Melodien hören und beurteilen, was Sie hören.
+Diese Aufgabe kann zunächst schwierig sein, besonders zu Beginn des Tests. Das ist völlig normal und zu erwarten. Bitte lassen Sie sich nicht entmutigen, wenn Sie bei den Antworten unsicher sind. Vertrauen Sie einfach auf Ihre beste Einschätzung.
+Bitte absolvieren Sie den Test in einer ruhigen Umgebung und verwenden Sie Kopfhörer oder Lautsprecher mit guter Klangqualität.</t>
+  </si>
+  <si>
+    <t>Du hast den Statistical Learning Test erfolgreich beendet.</t>
+  </si>
+  <si>
+    <t>Sie haben den Statistical Learning Test erfolgreich beendet.</t>
+  </si>
+  <si>
+    <t>You have completed the Statistical Learning Test.</t>
+  </si>
+  <si>
+    <t>Statistical Learning Test</t>
+  </si>
+  <si>
+    <t>On each trial, you will hear a short melody. Your task is to decide which of two groups the melody belongs to: Group A or Group B. Press the corresponding button to give your answer. After each response, you will receive feedback. 
+In the beginning, you will have to guess, but the feedback will help you to make better decisions as the test continues.
+Click the button below when you are ready to begin.</t>
+  </si>
+  <si>
+    <t>Bei jedem Durchgang hörst du eine kurze Melodie. Deine Aufgabe ist es zu entscheiden, zu welcher von zwei Gruppen die Melodie gehört: Gruppe A oder Gruppe B. Drücke die entsprechende Schaltfläche, um deine Antwort abzugeben. Nach jeder Antwort erhältst du eine Rückmeldung.
+Zu Beginn wirst du raten müssen, aber die Rückmeldungen werden dir helfen, im Verlauf des Tests bessere Entscheidungen zu treffen.
+Klicke auf den Button unten, wenn du bereit bist zu beginnen.</t>
+  </si>
+  <si>
+    <t>Bei jedem Durchgang hören Sie eine kurze Melodie. Ihre Aufgabe ist es zu entscheiden, zu welcher von zwei Gruppen die Melodie gehört: Gruppe A oder Gruppe B. Drücken Sie die entsprechende Schaltfläche, um Ihre Antwort abzugeben. Nach jeder Antwort erhalten Sie eine Rückmeldung.
+Zu Beginn werden Sie raten müssen, aber die Rückmeldungen werden Ihnen helfen, im Verlauf des Tests bessere Entscheidungen zu treffen.
+Klicken Sie auf die Schaltfläche unten, wenn Sie bereit sind zu beginnen.</t>
   </si>
   <si>
     <t>Du hast den ersten Block geschafft!
-Nun folgen nochmal 20 Melodien, die entweder von Komponistin 1 oder Komponistin 2 komponiert wurden.
+Nun folgen nochmal 24 Melodien, die entweder vonA oder B komponiert wurden.
 Entscheide intuitiv, wer welche Melodie komponiert hat.
 Achtung: Wenn Du eine Entscheidungsstrategie für den ersten Block hattest, gilt die für den nächsten Block nicht mehr!</t>
   </si>
   <si>
     <t>Sie haben den ersten Block geschafft!
-Nun folgen nochmal 20 Melodien, die entweder von Komponistin 1 oder Komponistin 2 komponiert wurden.
+Nun folgen nochmal 24 Melodien, die entweder von A oder B komponiert wurden.
 Entscheiden Sie intuitiv, wer welche Melodie komponiert hat.
 Achtung: Wenn Sie eine Entscheidungsstrategie für den ersten Block hatten, gilt die für den nächsten Block nicht mehr!</t>
   </si>
   <si>
     <t>You have completed the first block!
-Now you will hear another 20 melodies, each composed either by composer 1 or composer 2.
+Now you will hear another 24 melodies, each composed either by A or B.
 Decide intuitively who composed each melody.
 Caution: If you used a decision strategy in the first block, it will no longer apply in the next block!</t>
   </si>
   <si>
-    <t>Richtig, die Melodie stammt von Komponistin {{composer}}!</t>
-  </si>
-  <si>
-    <t>Richtig, die Melodie stammt von {{composer}}!</t>
-  </si>
-  <si>
-    <t>Falsch, die Melodie stammt von {{composer}}!</t>
-  </si>
-  <si>
-    <t>Correct, the melody was composed by {{composer}}!</t>
-  </si>
-  <si>
-    <t>False, the melody was composed by {{composer}}!</t>
-  </si>
-  <si>
-    <t>Falsch, die Melodie stammt von Komponistin {{composer}}!</t>
-  </si>
-  <si>
     <t>Du hast den zweiten Block geschafft!
-Nun folgen nochmal 20 Melodien, die entweder von Komponistin 1 oder Komponistin 2 komponiert wurden.
+Nun folgen nochmal 24 Melodien, die entweder vonA oder B komponiert wurden.
 Entscheide intuitiv, wer welche Melodie komponiert hat.
-Achtung: Wenn Du eine Entscheidungsstrategie für den zweiten Block hattest, gilt die für den nächsten Block nicht mehr!</t>
+Achtung: Wenn Du eine Entscheidungsstrategie für den ersten Block hattest, gilt die für den nächsten Block nicht mehr!</t>
   </si>
   <si>
     <t>Sie haben den zweiten Block geschafft!
-Nun folgen nochmal 20 Melodien, die entweder von Komponistin 1 oder Komponistin 2 komponiert wurden.
+Nun folgen nochmal 24 Melodien, die entweder von A oder B komponiert wurden.
 Entscheiden Sie intuitiv, wer welche Melodie komponiert hat.
-Achtung: Wenn Sie eine Entscheidungsstrategie für den zweiten Block hatten, gilt die für den nächsten Block nicht mehr!</t>
+Achtung: Wenn Sie eine Entscheidungsstrategie für den ersten Block hatten, gilt die für den nächsten Block nicht mehr!</t>
   </si>
   <si>
     <t>You have completed the second block!
-Now you will hear another 20 melodies, each composed either by composer 1 or composer 2.
+Now you will hear another 24 melodies, each composed either by A or B.
 Decide intuitively who composed each melody.
-Caution: If you used a decision strategy in the second block, it will no longer apply in the next block!</t>
-  </si>
-  <si>
-    <t>FINAL_FEEDBACK_BLOCK1</t>
-  </si>
-  <si>
-    <t>FINAL_FEEDBACK_BLOCK2</t>
-  </si>
-  <si>
-    <t>FINAL_FEEDBACK_BLOCK3</t>
-  </si>
-  <si>
-    <t>Im ersten Block hast Du {{number_correct_1}} Melodien richtig zugeordnet.</t>
-  </si>
-  <si>
-    <t>Im ersten Block haben Sie {{number_correct_1}} Melodien richtig zugeordnet.</t>
-  </si>
-  <si>
-    <t>In the first block, you identified {{number_correct_1}} melodies correctly.</t>
-  </si>
-  <si>
-    <t>Im zweiten Block hast Du {{number_correct_2}} Melodien richtig zugeordnet.</t>
-  </si>
-  <si>
-    <t>Im zweiten Block haben Sie {{number_correct_2}} Melodien richtig zugeordnet.</t>
-  </si>
-  <si>
-    <t>In the second block, you identified {{number_correct_2}} melodies correctly.</t>
-  </si>
-  <si>
-    <t>Im dritten Block hast Du {{number_correct_3}} Melodien richtig zugeordnet.</t>
-  </si>
-  <si>
-    <t>Im dritten Block haben Sie {{number_correct_3}} Melodien richtig zugeordnet.</t>
-  </si>
-  <si>
-    <t>In the third block, you identified {{number_correct_3}} melodies correctly.</t>
-  </si>
-  <si>
-    <t>In this study, we would like to measure your musical listening abilities. You will listen to short melodies and make judgements about what you hear.
-This task may feel difficult at first, especially at the beginning of the test. This is completely normal and expected. Please do not get discouraged if you are unsure about your answers, just go with your best guess and keep going.
-Please complete the test in a quiet environment using headphones or good-quality speakers.</t>
+Caution: If you used a decision strategy in the first block, it will no longer apply in the next block!</t>
   </si>
 </sst>
 </file>
@@ -815,13 +814,13 @@
         <v>3</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>61</v>
+        <v>89</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>61</v>
+        <v>89</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>62</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="213.75" x14ac:dyDescent="0.45">
@@ -829,13 +828,13 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>63</v>
+        <v>91</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>64</v>
+        <v>92</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
@@ -871,13 +870,13 @@
         <v>7</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.45">
@@ -913,13 +912,13 @@
         <v>10</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.45">
@@ -969,13 +968,13 @@
         <v>14</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>68</v>
+        <v>93</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>69</v>
+        <v>94</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>70</v>
+        <v>95</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.45">
@@ -983,13 +982,13 @@
         <v>15</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>71</v>
+        <v>96</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>71</v>
+        <v>96</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>72</v>
+        <v>96</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="42.75" x14ac:dyDescent="0.45">
@@ -1048,18 +1047,18 @@
         <v>41</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="156.75" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:4" ht="199.5" x14ac:dyDescent="0.45">
       <c r="A19" s="2" t="s">
         <v>42</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.45">
@@ -1106,104 +1105,105 @@
     </row>
     <row r="23" spans="1:4" ht="156.75" x14ac:dyDescent="0.45">
       <c r="A23" s="1" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="171" x14ac:dyDescent="0.45">
       <c r="A24" s="1" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A25" s="1" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>88</v>
+        <v>73</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A26" s="1" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>87</v>
+        <v>72</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>89</v>
+        <v>74</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A27" s="1" t="s">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>97</v>
+        <v>79</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>99</v>
+        <v>81</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A28" s="1" t="s">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A29" s="1" t="s">
-        <v>96</v>
+        <v>78</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>104</v>
+        <v>86</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>105</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added an instruction page to the SLT
</commit_message>
<xml_diff>
--- a/data_raw/SLT_dict.xlsx
+++ b/data_raw/SLT_dict.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anton\Nextcloud\Promotion\Tests\SLT\data_raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F8D822A-3DAA-42D0-867A-13709147C462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56D7B60E-AF2E-4FAD-84A6-615A3A524EF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="17115" windowHeight="10755" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="123">
   <si>
     <t>key</t>
   </si>
@@ -368,16 +368,76 @@
 Now you will hear another 24 melodies, each composed either by A or B.
 Decide intuitively who composed each melody.
 Caution: If you used a decision strategy in the first block, it will no longer apply in the next block!</t>
+  </si>
+  <si>
+    <t>DEMO_INTRO</t>
+  </si>
+  <si>
+    <t>On each trial, you will hear a short melody. Your task is to decide which of two groups the melody belongs to: Group A or Group B. Press the corresponding button to give your answer. After each response, you will receive feedback. Click the button below when you are ready to begin.</t>
+  </si>
+  <si>
+    <t>Bei jedem Durchgang hörst du eine kurze Melodie. Deine Aufgabe ist es zu entscheiden, zu welcher von zwei Gruppen die Melodie gehört: Gruppe A oder Gruppe B. Drücke die entsprechende Schaltfläche, um deine Antwort abzugeben. Nach jeder Antwort erhältst du eine Rückmeldung.
+Klicke auf die Schaltfläche unten, wenn du bereit bist zu beginnen.</t>
+  </si>
+  <si>
+    <t>Bei jedem Durchgang hören Sie eine kurze Melodie. Ihre Aufgabe ist es zu entscheiden, zu welcher von zwei Gruppen die Melodie gehört: Gruppe A oder Gruppe B. Drücken Sie die entsprechende Schaltfläche, um Ihre Antwort abzugeben. Nach jeder Antwort erhalten Sie eine Rückmeldung.
+Klicken Sie auf die Schaltfläche unten, wenn Sie bereit sind zu beginnen.</t>
+  </si>
+  <si>
+    <t>DEMO_ITEM_A</t>
+  </si>
+  <si>
+    <t>Listen to this example melody from Group A.</t>
+  </si>
+  <si>
+    <t>Höre dir diese Beispielmelodie von A an.</t>
+  </si>
+  <si>
+    <t>Hören Sie sich diese Beispielmelodie von A an.</t>
+  </si>
+  <si>
+    <t>DEMO_ITEM_B</t>
+  </si>
+  <si>
+    <t>Höre dir diese Beispielmelodie von B an.</t>
+  </si>
+  <si>
+    <t>Hören Sie sich diese Beispielmelodie von B an.</t>
+  </si>
+  <si>
+    <t>Listen to this example melody from Group B.</t>
+  </si>
+  <si>
+    <t>Now the real test begins. The melodies might sound different from the ones in the demo. Don't worry if the task feels very difficult at first, this is completely normal. You will receive feedback after each trial.</t>
+  </si>
+  <si>
+    <t>Jetzt beginnt der eigentliche Test. Die Melodien können anders klingen als die im Übungsdurchgang. Mach dir keine Sorgen, wenn die Aufgabe anfangs sehr schwierig erscheint, das ist völlig normal. Nach jedem Durchgang erhältst du eine Rückmeldung.</t>
+  </si>
+  <si>
+    <t>Jetzt beginnt der eigentliche Test. Die Melodien können anders klingen als die im Übungsdurchgang. Machen Sie sich keine Sorgen, wenn die Aufgabe anfangs sehr schwierig erscheint, das ist völlig normal. Nach jedem Durchgang erhalten Sie eine Rückmeldung.</t>
+  </si>
+  <si>
+    <t>DEMO_OUTRO</t>
+  </si>
+  <si>
+    <t>CORRECT_B</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -403,7 +463,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -411,6 +471,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -786,7 +850,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="26.3984375" style="1" customWidth="1"/>
@@ -1201,6 +1265,76 @@
         <v>87</v>
       </c>
     </row>
+    <row r="30" spans="1:4" ht="128.25" x14ac:dyDescent="0.45">
+      <c r="A30" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A31" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A32" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="85.5" x14ac:dyDescent="0.45">
+      <c r="A33" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A34" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
changed wording in dict
</commit_message>
<xml_diff>
--- a/data_raw/SLT_dict.xlsx
+++ b/data_raw/SLT_dict.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anton\Nextcloud\Promotion\Tests\SLT\data_raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{599A41BD-0EF6-4103-957C-24C427BAC2AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37EE9C65-A495-4DC5-B83C-92AEE7E244C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="17115" windowHeight="10755" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22450" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EDT" sheetId="1" r:id="rId1"/>
@@ -292,21 +292,6 @@
     <t>Willkommen zum Statistical Learning Test</t>
   </si>
   <si>
-    <t>In this test, we would like to measure your musical listening abilities. You will listen to short melodies and make judgements about what you hear.
-This task may feel difficult at first, especially at the beginning of the test. This is completely normal and expected. Please do not get discouraged if you are unsure about your answers, just go with your best guess and keep going.
-Please complete the test in a quiet environment using headphones or good-quality speakers.</t>
-  </si>
-  <si>
-    <t>In dieser Studie möchten wir deine  musikalische Hörfähigkeit messen. Du wirst kurze Melodien hören und beurteilen, was du hörst.
-Diese Aufgabe kann zunächst schwierig sein, besonders zu Beginn des Tests. Das ist völlig normal und zu erwarten. Bitte lass dich nicht entmutigen, wenn du bei deinen Antworten unsicher bist. Vertraue einfach auf deine beste Einschätzung.
-Bitte absolviere den Test in einer ruhigen Umgebung und verwende Kopfhörer oder Lautsprecher mit guter Klangqualität.</t>
-  </si>
-  <si>
-    <t>In dieser Studie möchten wir Ihre  musikalische Hörfähigkeit messen. Sie werden kurze Melodien hören und beurteilen, was Sie hören.
-Diese Aufgabe kann zunächst schwierig sein, besonders zu Beginn des Tests. Das ist völlig normal und zu erwarten. Bitte lassen Sie sich nicht entmutigen, wenn Sie bei den Antworten unsicher sind. Vertrauen Sie einfach auf Ihre beste Einschätzung.
-Bitte absolvieren Sie den Test in einer ruhigen Umgebung und verwenden Sie Kopfhörer oder Lautsprecher mit guter Klangqualität.</t>
-  </si>
-  <si>
     <t>Du hast den Statistical Learning Test erfolgreich beendet.</t>
   </si>
   <si>
@@ -332,24 +317,6 @@
     <t>Bei jedem Durchgang hören Sie eine kurze Melodie. Ihre Aufgabe ist es zu entscheiden, zu welcher von zwei Gruppen die Melodie gehört: Gruppe A oder Gruppe B. Drücken Sie die entsprechende Schaltfläche, um Ihre Antwort abzugeben. Nach jeder Antwort erhalten Sie eine Rückmeldung.
 Zu Beginn werden Sie raten müssen, aber die Rückmeldungen werden Ihnen helfen, im Verlauf des Tests bessere Entscheidungen zu treffen.
 Klicken Sie auf die Schaltfläche unten, wenn Sie bereit sind zu beginnen.</t>
-  </si>
-  <si>
-    <t>Du hast den ersten Block geschafft!
-Nun folgen nochmal 24 Melodien, die entweder vonA oder B komponiert wurden.
-Entscheide intuitiv, wer welche Melodie komponiert hat.
-Achtung: Wenn Du eine Entscheidungsstrategie für den ersten Block hattest, gilt die für den nächsten Block nicht mehr!</t>
-  </si>
-  <si>
-    <t>Sie haben den ersten Block geschafft!
-Nun folgen nochmal 24 Melodien, die entweder von A oder B komponiert wurden.
-Entscheiden Sie intuitiv, wer welche Melodie komponiert hat.
-Achtung: Wenn Sie eine Entscheidungsstrategie für den ersten Block hatten, gilt die für den nächsten Block nicht mehr!</t>
-  </si>
-  <si>
-    <t>You have completed the first block!
-Now you will hear another 24 melodies, each composed either by A or B.
-Decide intuitively who composed each melody.
-Caution: If you used a decision strategy in the first block, it will no longer apply in the next block!</t>
   </si>
   <si>
     <t>Du hast den zweiten Block geschafft!
@@ -433,6 +400,39 @@
   </si>
   <si>
     <t>Practice: Decide whether this melody belongs to Group A or Group B.</t>
+  </si>
+  <si>
+    <t>In this test, we would like to measure your musical listening abilities. You will listen to short melodies and make judgements about what you hear.
+This task may feel difficult at first, especially at the beginning of the test. This is completely normal and expected. Please do not get discouraged if you are unsure about your answers, just go with your best guess, learn with the feedback and keep going.
+Please complete the test in a quiet environment using headphones or good-quality speakers.</t>
+  </si>
+  <si>
+    <t>You have completed the first block!
+Now you will hear another 24 melodies, each composed either by A or B.
+Decide intuitively who composed each melody.
+Caution: If you used a decision strategy in the previous block, it will no longer apply in the next block!</t>
+  </si>
+  <si>
+    <t>Sie haben den ersten Block geschafft!
+Nun folgen nochmal 24 Melodien, die entweder von A oder B komponiert wurden.
+Entscheiden Sie intuitiv, wer welche Melodie komponiert hat.
+Achtung: Wenn Sie eine Entscheidungsstrategie für den vorherigen Block hatten, gilt die für den nächsten Block nicht mehr!</t>
+  </si>
+  <si>
+    <t>Du hast den ersten Block geschafft!
+Nun folgen nochmal 24 Melodien, die entweder vonA oder B komponiert wurden.
+Entscheide intuitiv, wer welche Melodie komponiert hat.
+Achtung: Wenn Du eine Entscheidungsstrategie für den vorherigen Block hattest, gilt die für den nächsten Block nicht mehr!</t>
+  </si>
+  <si>
+    <t>In dieser Studie möchten wir Ihre  musikalische Hörfähigkeit messen. Sie werden kurze Melodien hören und beurteilen, was Sie hören.
+Diese Aufgabe kann zunächst schwierig sein, besonders zu Beginn des Tests. Das ist völlig normal und zu erwarten. Bitte lassen Sie sich nicht entmutigen, wenn Sie bei den Antworten unsicher sind. Nutzen Sie das Feedback und vertrauen Sie einfach auf Ihre beste Einschätzung.
+Bitte absolvieren Sie den Test in einer ruhigen Umgebung und verwenden Sie Kopfhörer oder Lautsprecher mit guter Klangqualität.</t>
+  </si>
+  <si>
+    <t>In dieser Studie möchten wir deine  musikalische Hörfähigkeit messen. Du wirst kurze Melodien hören und beurteilen, was du hörst.
+Diese Aufgabe kann zunächst schwierig sein, besonders zu Beginn des Tests. Das ist völlig normal und zu erwarten. Bitte lass dich nicht entmutigen, wenn du bei deinen Antworten unsicher bist. Nutze das Feedback und vertraue einfach auf deine beste Einschätzung.
+Bitte absolviere den Test in einer ruhigen Umgebung und verwende Kopfhörer oder Lautsprecher mit guter Klangqualität.</t>
   </si>
 </sst>
 </file>
@@ -515,9 +515,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>203200</xdr:colOff>
+      <xdr:colOff>204787</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>225926</xdr:rowOff>
+      <xdr:rowOff>222750</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -899,18 +899,18 @@
         <v>88</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="213.75" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:4" ht="256.5" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>91</v>
+        <v>126</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>92</v>
+        <v>125</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>90</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
@@ -1044,13 +1044,13 @@
         <v>14</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.45">
@@ -1058,13 +1058,13 @@
         <v>15</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="42.75" x14ac:dyDescent="0.45">
@@ -1128,13 +1128,13 @@
         <v>42</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.45">
@@ -1184,13 +1184,13 @@
         <v>66</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>100</v>
+        <v>124</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>101</v>
+        <v>123</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>102</v>
+        <v>122</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="171" x14ac:dyDescent="0.45">
@@ -1198,13 +1198,13 @@
         <v>67</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
@@ -1279,63 +1279,63 @@
     </row>
     <row r="30" spans="1:4" ht="128.25" x14ac:dyDescent="0.45">
       <c r="A30" s="1" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A31" s="1" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A32" s="1" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A33" s="1" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A34" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>71</v>
@@ -1349,16 +1349,16 @@
     </row>
     <row r="35" spans="1:4" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A35" s="1" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changed text and buttons to specific composer names
</commit_message>
<xml_diff>
--- a/data_raw/SLT_dict.xlsx
+++ b/data_raw/SLT_dict.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anton\Nextcloud\Promotion\Tests\SLT\data_raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anton\Nextcloud\Promotion\Tests\SLT_v3\SLT3\data_raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4925B71-793B-473D-AB4B-2DEF80D0C900}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ADF64D6-7D7C-45CD-A5BB-230DEECA9040}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="72120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="17115" windowHeight="10755" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EDT" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="143">
   <si>
     <t>key</t>
   </si>
@@ -319,56 +319,15 @@
 Klicken Sie auf die Schaltfläche unten, wenn Sie bereit sind zu beginnen.</t>
   </si>
   <si>
-    <t>Du hast den zweiten Block geschafft!
-Nun folgen nochmal 24 Melodien, die entweder vonA oder B komponiert wurden.
-Entscheide intuitiv, wer welche Melodie komponiert hat.
-Achtung: Wenn Du eine Entscheidungsstrategie für den ersten Block hattest, gilt die für den nächsten Block nicht mehr!</t>
-  </si>
-  <si>
-    <t>Sie haben den zweiten Block geschafft!
-Nun folgen nochmal 24 Melodien, die entweder von A oder B komponiert wurden.
-Entscheiden Sie intuitiv, wer welche Melodie komponiert hat.
-Achtung: Wenn Sie eine Entscheidungsstrategie für den ersten Block hatten, gilt die für den nächsten Block nicht mehr!</t>
-  </si>
-  <si>
     <t>DEMO_INTRO</t>
   </si>
   <si>
-    <t>On each trial, you will hear a short melody. Your task is to decide which of two groups the melody belongs to: Group A or Group B. Press the corresponding button to give your answer. After each response, you will receive feedback. Click the button below when you are ready to begin.</t>
-  </si>
-  <si>
-    <t>Bei jedem Durchgang hörst du eine kurze Melodie. Deine Aufgabe ist es zu entscheiden, zu welcher von zwei Gruppen die Melodie gehört: Gruppe A oder Gruppe B. Drücke die entsprechende Schaltfläche, um deine Antwort abzugeben. Nach jeder Antwort erhältst du eine Rückmeldung.
-Klicke auf die Schaltfläche unten, wenn du bereit bist zu beginnen.</t>
-  </si>
-  <si>
-    <t>Bei jedem Durchgang hören Sie eine kurze Melodie. Ihre Aufgabe ist es zu entscheiden, zu welcher von zwei Gruppen die Melodie gehört: Gruppe A oder Gruppe B. Drücken Sie die entsprechende Schaltfläche, um Ihre Antwort abzugeben. Nach jeder Antwort erhalten Sie eine Rückmeldung.
-Klicken Sie auf die Schaltfläche unten, wenn Sie bereit sind zu beginnen.</t>
-  </si>
-  <si>
     <t>DEMO_ITEM_A</t>
   </si>
   <si>
-    <t>Listen to this example melody from Group A.</t>
-  </si>
-  <si>
-    <t>Höre dir diese Beispielmelodie von A an.</t>
-  </si>
-  <si>
-    <t>Hören Sie sich diese Beispielmelodie von A an.</t>
-  </si>
-  <si>
     <t>DEMO_ITEM_B</t>
   </si>
   <si>
-    <t>Höre dir diese Beispielmelodie von B an.</t>
-  </si>
-  <si>
-    <t>Hören Sie sich diese Beispielmelodie von B an.</t>
-  </si>
-  <si>
-    <t>Listen to this example melody from Group B.</t>
-  </si>
-  <si>
     <t>Now the real test begins. The melodies might sound different from the ones in the demo. Don't worry if the task feels very difficult at first, this is completely normal. You will receive feedback after each trial.</t>
   </si>
   <si>
@@ -385,15 +344,6 @@
   </si>
   <si>
     <t>DEMO_TRIAL_INSTRUCTION</t>
-  </si>
-  <si>
-    <t>Übung: Entscheide, ob diese Melodie von Gruppe A oder Gruppe B stammt.</t>
-  </si>
-  <si>
-    <t>Übung: Entscheiden Sie, ob diese Melodie von Gruppe A oder Gruppe B stammt.</t>
-  </si>
-  <si>
-    <t>Practice: Decide whether this melody belongs to Group A or Group B.</t>
   </si>
   <si>
     <t>In this test, we would like to measure your musical listening abilities. You will listen to short melodies and make judgements about what you hear.
@@ -401,24 +351,6 @@
 Please complete the test in a quiet environment using headphones or good-quality speakers.</t>
   </si>
   <si>
-    <t>You have completed the first block!
-Now you will hear another 24 melodies, each composed either by A or B.
-Decide intuitively who composed each melody.
-Caution: If you used a decision strategy in the previous block, it will no longer apply in the next block!</t>
-  </si>
-  <si>
-    <t>Sie haben den ersten Block geschafft!
-Nun folgen nochmal 24 Melodien, die entweder von A oder B komponiert wurden.
-Entscheiden Sie intuitiv, wer welche Melodie komponiert hat.
-Achtung: Wenn Sie eine Entscheidungsstrategie für den vorherigen Block hatten, gilt die für den nächsten Block nicht mehr!</t>
-  </si>
-  <si>
-    <t>Du hast den ersten Block geschafft!
-Nun folgen nochmal 24 Melodien, die entweder vonA oder B komponiert wurden.
-Entscheide intuitiv, wer welche Melodie komponiert hat.
-Achtung: Wenn Du eine Entscheidungsstrategie für den vorherigen Block hattest, gilt die für den nächsten Block nicht mehr!</t>
-  </si>
-  <si>
     <t>In dieser Studie möchten wir Ihre  musikalische Hörfähigkeit messen. Sie werden kurze Melodien hören und beurteilen, was Sie hören.
 Diese Aufgabe kann zunächst schwierig sein, besonders zu Beginn des Tests. Das ist völlig normal und zu erwarten. Bitte lassen Sie sich nicht entmutigen, wenn Sie bei den Antworten unsicher sind. Nutzen Sie das Feedback und vertrauen Sie einfach auf Ihre beste Einschätzung.
 Bitte absolvieren Sie den Test in einer ruhigen Umgebung und verwenden Sie Kopfhörer oder Lautsprecher mit guter Klangqualität.</t>
@@ -429,10 +361,108 @@
 Bitte absolviere den Test in einer ruhigen Umgebung und verwende Kopfhörer oder Lautsprecher mit guter Klangqualität.</t>
   </si>
   <si>
-    <t>You have completed the second block!
-Now you will hear another 24 melodies, each composed either by A or B.
-Decide intuitively who composed each melody.
-Caution: If you used a decision strategy in the previous block, it will no longer apply in the next block!</t>
+    <t>CORRECT_COMPOSER</t>
+  </si>
+  <si>
+    <t>Richtig, diese Melodie wurde von {{composer}} komponiert.</t>
+  </si>
+  <si>
+    <t>Correct, this melody was composed by {{composer}}.</t>
+  </si>
+  <si>
+    <t>FALSE_COMPOSER</t>
+  </si>
+  <si>
+    <t>Falsch, diese Melodie wurde von {{composer}} komponiert.</t>
+  </si>
+  <si>
+    <t>False, this melody was composed by {{composer}}.</t>
+  </si>
+  <si>
+    <t>BLOCK1_INTRO</t>
+  </si>
+  <si>
+    <t>Bei jedem Durchgang hörst du eine kurze Melodie. Deine Aufgabe ist es zu entscheiden, wer von zwei Komponist*innen die Melodie geschrieben hat. Drücke die entsprechende Schaltfläche, um deine Antwort abzugeben. Nach jeder Antwort erhältst du eine Rückmeldung.
+Klicke auf die Schaltfläche unten, wenn du bereit bist zu beginnen.</t>
+  </si>
+  <si>
+    <t>Bei jedem Durchgang hören Sie eine kurze Melodie. Ihre Aufgabe ist es zu entscheiden,wer von zwei Komponist*innen die Melodie geschrieben hat. Drücken Sie die entsprechende Schaltfläche, um Ihre Antwort abzugeben. Nach jeder Antwort erhalten Sie eine Rückmeldung.
+Klicken Sie auf die Schaltfläche unten, wenn Sie bereit sind zu beginnen.</t>
+  </si>
+  <si>
+    <t>On each trial, you will hear a short melody. Your task is to decide which of two composers wrote the melody. Press the corresponding button to give your answer. After each response, you will receive feedback. Click the button below when you are ready to begin.</t>
+  </si>
+  <si>
+    <t>Höre dir diese Beispielmelodie an.</t>
+  </si>
+  <si>
+    <t>Hören Sie sich diese Beispielmelodie.</t>
+  </si>
+  <si>
+    <t>Listen to this example melody.</t>
+  </si>
+  <si>
+    <t>COMPOSER_A</t>
+  </si>
+  <si>
+    <t>Komponist*in A</t>
+  </si>
+  <si>
+    <t>Komponist*in B</t>
+  </si>
+  <si>
+    <t>Composer A</t>
+  </si>
+  <si>
+    <t>Composer B</t>
+  </si>
+  <si>
+    <t>COMPOSER_B</t>
+  </si>
+  <si>
+    <t>Hör dir diese Beispielmelodie an. Wer hat diese Melodie komponiert?</t>
+  </si>
+  <si>
+    <t>Hören Sie sich diese Beispielmelodie an. Wer hat diese Melodie komponiert?</t>
+  </si>
+  <si>
+    <t>Listen to this example melody. Who composed this melody?</t>
+  </si>
+  <si>
+    <t>DEMO_CORRECT</t>
+  </si>
+  <si>
+    <t>DEMO_FALSE</t>
+  </si>
+  <si>
+    <t>False.</t>
+  </si>
+  <si>
+    <t>In diesem Block hörst du Melodien von zwei Komponist*innen: **{{composer_a}}** und **{{composer_b}}**. \\ Entscheide intuitiv, wer jede Melodie komponiert hat. Am Anfang wirst du raten müssen. Nutze das Feedback, um dich zu verbessern.</t>
+  </si>
+  <si>
+    <t>In diesem Block hören Sie Melodien von zwei Komponist*innen: **{{composer_a}}** und **{{composer_b}}**.\\ Entscheiden Sie intuitiv, wer jede Melodie komponiert hat. Am Anfang werden Sie raten müssen.  Nutzen Sie das Feedback, um sich zu verbessern.</t>
+  </si>
+  <si>
+    <t>Gut gemacht! Du hast die erste Runde abgeschlossen. In der nächsten Runde hörst du Melodien von zwei neuen Komponist*innen: **{{composer_a}}** und **{{composer_b}}**. Versuche herauszufinden, welche Melodie zu wem gehört. \\ Drücke Weiter, wenn du bereit bist.</t>
+  </si>
+  <si>
+    <t>Gut gemacht! Sie haben die erste Runde abgeschlossen. In der nächsten Runde hören Sie Melodien von zwei neuen Komponist*innen: **{{composer_a}}** und **{{composer_b}}**. Versuche herauszufinden, welche Melodie zu wem gehört. \\ Drücken Sie Weiter, wenn Sie bereit sind.</t>
+  </si>
+  <si>
+    <t>Well done! You have completed the first round. In the next round, you will hear melodies by two new composers: **{{composer_a}}** and **{{composer_b}}**. Try to figure out which melody belongs to which composer. \\ Press Continue when you are ready.</t>
+  </si>
+  <si>
+    <t>Great work! Now for the final round  featuring two more composers: **{{composer_a}}** and **{{composer_b}}**.  \\ Press Continue when you are ready.</t>
+  </si>
+  <si>
+    <t>Super! Jetzt folgt die letzte Runde mit zwei weiteren Komponist*innen: **{{composer_a}}** und **{{composer_b}}**. \\  Drücken Sie Weiter, wenn Sie bereit sind.</t>
+  </si>
+  <si>
+    <t>Super! Jetzt folgt die letzte Runde mit zwei weiteren Komponist*innen: **{{composer_a}}** und **{{composer_b}}**. \\  Drücke Weiter, wenn du bereit bist.</t>
+  </si>
+  <si>
+    <t>In this block, you will listen to melodies by two composers: **{{composer_a}}** and **{{composer_b}}**. \\ Decide intuitively who composed each melody. In the beginning, you will have to guess. Use the feedback to improve over time.</t>
   </si>
 </sst>
 </file>
@@ -543,7 +573,7 @@
         <a:noFill/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:solidFill>
                 <a:srgbClr val="FFFFFF"/>
               </a:solidFill>
@@ -862,7 +892,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="26.3984375" style="1" customWidth="1"/>
@@ -904,13 +934,13 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>125</v>
+        <v>108</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>120</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
@@ -1179,32 +1209,32 @@
         <v>51</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="156.75" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:4" ht="114" x14ac:dyDescent="0.45">
       <c r="A23" s="1" t="s">
         <v>66</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>122</v>
+        <v>137</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="171" x14ac:dyDescent="0.45">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="71.25" x14ac:dyDescent="0.45">
       <c r="A24" s="1" t="s">
         <v>67</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>97</v>
+        <v>141</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>98</v>
+        <v>140</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
@@ -1277,65 +1307,65 @@
         <v>87</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:4" ht="114" x14ac:dyDescent="0.45">
       <c r="A30" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A31" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A32" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="D30" s="3" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A31" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A32" s="1" t="s">
-        <v>107</v>
-      </c>
       <c r="B32" s="4" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>110</v>
+        <v>121</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A33" s="1" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A34" s="1" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>71</v>
@@ -1347,18 +1377,116 @@
         <v>73</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A35" s="1" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>119</v>
+        <v>130</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A36" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B36" t="s">
+        <v>110</v>
+      </c>
+      <c r="C36" t="s">
+        <v>110</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A37" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B37" t="s">
+        <v>113</v>
+      </c>
+      <c r="C37" t="s">
+        <v>113</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="114" x14ac:dyDescent="0.45">
+      <c r="A38" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A39" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A40" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A41" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A42" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>133</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changed feedback. modified brake pages
</commit_message>
<xml_diff>
--- a/data_raw/SLT_dict.xlsx
+++ b/data_raw/SLT_dict.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anton\Nextcloud\Promotion\Tests\SLT_v3\SLT3\data_raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anton\Nextcloud\Promotion\Tests\SLT\data_raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ADF64D6-7D7C-45CD-A5BB-230DEECA9040}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{777569FF-8AEC-4D9E-8A53-B8D2625C002E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="17115" windowHeight="10755" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="145">
   <si>
     <t>key</t>
   </si>
@@ -257,51 +257,6 @@
   </si>
   <si>
     <t>FINAL_FEEDBACK_BLOCK3</t>
-  </si>
-  <si>
-    <t>Im ersten Block hast Du {{number_correct_1}} Melodien richtig zugeordnet.</t>
-  </si>
-  <si>
-    <t>Im ersten Block haben Sie {{number_correct_1}} Melodien richtig zugeordnet.</t>
-  </si>
-  <si>
-    <t>In the first block, you identified {{number_correct_1}} melodies correctly.</t>
-  </si>
-  <si>
-    <t>Im zweiten Block hast Du {{number_correct_2}} Melodien richtig zugeordnet.</t>
-  </si>
-  <si>
-    <t>Im zweiten Block haben Sie {{number_correct_2}} Melodien richtig zugeordnet.</t>
-  </si>
-  <si>
-    <t>In the second block, you identified {{number_correct_2}} melodies correctly.</t>
-  </si>
-  <si>
-    <t>Im dritten Block hast Du {{number_correct_3}} Melodien richtig zugeordnet.</t>
-  </si>
-  <si>
-    <t>Im dritten Block haben Sie {{number_correct_3}} Melodien richtig zugeordnet.</t>
-  </si>
-  <si>
-    <t>In the third block, you identified {{number_correct_3}} melodies correctly.</t>
-  </si>
-  <si>
-    <t>Welcome to the Statistical Learning Test</t>
-  </si>
-  <si>
-    <t>Willkommen zum Statistical Learning Test</t>
-  </si>
-  <si>
-    <t>Du hast den Statistical Learning Test erfolgreich beendet.</t>
-  </si>
-  <si>
-    <t>Sie haben den Statistical Learning Test erfolgreich beendet.</t>
-  </si>
-  <si>
-    <t>You have completed the Statistical Learning Test.</t>
-  </si>
-  <si>
-    <t>Statistical Learning Test</t>
   </si>
   <si>
     <t>On each trial, you will hear a short melody. Your task is to decide which of two groups the melody belongs to: Group A or Group B. Press the corresponding button to give your answer. After each response, you will receive feedback. 
@@ -346,11 +301,6 @@
     <t>DEMO_TRIAL_INSTRUCTION</t>
   </si>
   <si>
-    <t>In this test, we would like to measure your musical listening abilities. You will listen to short melodies and make judgements about what you hear.
-This task may feel difficult at first, especially at the beginning of the test. This is completely normal and expected. Please do not get discouraged if you are unsure about your answers, just go with your best guess, learn with the feedback and keep going.
-Please complete the test in a quiet environment using headphones or good-quality speakers.</t>
-  </si>
-  <si>
     <t>In dieser Studie möchten wir Ihre  musikalische Hörfähigkeit messen. Sie werden kurze Melodien hören und beurteilen, was Sie hören.
 Diese Aufgabe kann zunächst schwierig sein, besonders zu Beginn des Tests. Das ist völlig normal und zu erwarten. Bitte lassen Sie sich nicht entmutigen, wenn Sie bei den Antworten unsicher sind. Nutzen Sie das Feedback und vertrauen Sie einfach auf Ihre beste Einschätzung.
 Bitte absolvieren Sie den Test in einer ruhigen Umgebung und verwenden Sie Kopfhörer oder Lautsprecher mit guter Klangqualität.</t>
@@ -438,31 +388,87 @@
     <t>False.</t>
   </si>
   <si>
-    <t>In diesem Block hörst du Melodien von zwei Komponist*innen: **{{composer_a}}** und **{{composer_b}}**. \\ Entscheide intuitiv, wer jede Melodie komponiert hat. Am Anfang wirst du raten müssen. Nutze das Feedback, um dich zu verbessern.</t>
-  </si>
-  <si>
-    <t>In diesem Block hören Sie Melodien von zwei Komponist*innen: **{{composer_a}}** und **{{composer_b}}**.\\ Entscheiden Sie intuitiv, wer jede Melodie komponiert hat. Am Anfang werden Sie raten müssen.  Nutzen Sie das Feedback, um sich zu verbessern.</t>
-  </si>
-  <si>
-    <t>Gut gemacht! Du hast die erste Runde abgeschlossen. In der nächsten Runde hörst du Melodien von zwei neuen Komponist*innen: **{{composer_a}}** und **{{composer_b}}**. Versuche herauszufinden, welche Melodie zu wem gehört. \\ Drücke Weiter, wenn du bereit bist.</t>
-  </si>
-  <si>
-    <t>Gut gemacht! Sie haben die erste Runde abgeschlossen. In der nächsten Runde hören Sie Melodien von zwei neuen Komponist*innen: **{{composer_a}}** und **{{composer_b}}**. Versuche herauszufinden, welche Melodie zu wem gehört. \\ Drücken Sie Weiter, wenn Sie bereit sind.</t>
-  </si>
-  <si>
-    <t>Well done! You have completed the first round. In the next round, you will hear melodies by two new composers: **{{composer_a}}** and **{{composer_b}}**. Try to figure out which melody belongs to which composer. \\ Press Continue when you are ready.</t>
-  </si>
-  <si>
-    <t>Great work! Now for the final round  featuring two more composers: **{{composer_a}}** and **{{composer_b}}**.  \\ Press Continue when you are ready.</t>
-  </si>
-  <si>
-    <t>Super! Jetzt folgt die letzte Runde mit zwei weiteren Komponist*innen: **{{composer_a}}** und **{{composer_b}}**. \\  Drücken Sie Weiter, wenn Sie bereit sind.</t>
-  </si>
-  <si>
-    <t>Super! Jetzt folgt die letzte Runde mit zwei weiteren Komponist*innen: **{{composer_a}}** und **{{composer_b}}**. \\  Drücke Weiter, wenn du bereit bist.</t>
-  </si>
-  <si>
-    <t>In this block, you will listen to melodies by two composers: **{{composer_a}}** and **{{composer_b}}**. \\ Decide intuitively who composed each melody. In the beginning, you will have to guess. Use the feedback to improve over time.</t>
+    <t>Willkommen zum Statistical Melody Learning Test</t>
+  </si>
+  <si>
+    <t>Welcome to the Statistical Melody Learning Test</t>
+  </si>
+  <si>
+    <t>Willkommen zum Melodielerntest</t>
+  </si>
+  <si>
+    <t>Du hast den Melodielerntest erfolgreich beendet.</t>
+  </si>
+  <si>
+    <t>Sie haben den Statistical Melody Learning Test erfolgreich beendet.</t>
+  </si>
+  <si>
+    <t>You have completed the Statistical Melody Learning Test.</t>
+  </si>
+  <si>
+    <t>Melodielerntest</t>
+  </si>
+  <si>
+    <t>Statistical Melody Learning Test</t>
+  </si>
+  <si>
+    <t>In this test, we would like to measure your musical listening abilities. You will listen to short melodies and make judgements about what you hear.
+This task may feel difficult at first, especially at the beginning of the test. This is completely normal and expected. Please do not get discouraged if you are unsure about your answers, just go with your best guess, learn from the feedback and keep going.
+Please complete the test in a quiet environment using headphones or good-quality speakers.</t>
+  </si>
+  <si>
+    <t>In the first block, you identified {{number_correct_1}} out of {{total_1}} melodies correctly ({{percent_1}}%).</t>
+  </si>
+  <si>
+    <t>Im ersten Block haben Sie {{number_correct_1}} von {{total_1}} Melodien richtig zugeordnet ({{percent_1}}%).</t>
+  </si>
+  <si>
+    <t>Im ersten Block hast Du {{number_correct_1}} von {{total_1}} Melodien richtig zugeordnet ({{percent_1}}%).</t>
+  </si>
+  <si>
+    <t>Im zweiten Block hast Du {{number_correct_2}} von {{total_2}} Melodien richtig zugeordnet ({{percent_2}}%).</t>
+  </si>
+  <si>
+    <t>Im zweiten Block haben Sie  {{number_correct_2}} von {{total_2}} Melodien richtig zugeordnet ({{percent_2}}%).</t>
+  </si>
+  <si>
+    <t>Im dritten Block hast Du {{number_correct_3}} von {{total_3}} Melodien richtig zugeordnet ({{percent_3}}%).</t>
+  </si>
+  <si>
+    <t>Im dritten Block haben Sie {{number_correct_3}} von {{total_3}} Melodien richtig zugeordnet ({{percent_3}}%).</t>
+  </si>
+  <si>
+    <t>In the second block, you identified {{number_correct_2}} out of {{total_2}} melodies correctly ({{percent_2}}%).</t>
+  </si>
+  <si>
+    <t>In the third block, you identified {{number_correct_3}} out of {{total_3}} melodies correctly ({{percent_3}}%).</t>
+  </si>
+  <si>
+    <t>Gut gemacht! Du hast die erste Runde abgeschlossen. In der nächsten Runde hörst du {{num_items}} Melodien von zwei neuen Komponist*innen: **{{composer_a}}** und **{{composer_b}}**. Versuche herauszufinden, welche Melodie zu wem gehört. \\ Drücke Weiter, wenn du bereit bist.</t>
+  </si>
+  <si>
+    <t>Gut gemacht! Sie haben die erste Runde abgeschlossen. In der nächsten Runde hören Sie {{num_items}} Melodien von zwei neuen Komponist*innen: **{{composer_a}}** und **{{composer_b}}**. Versuche herauszufinden, welche Melodie zu wem gehört. \\ Drücken Sie Weiter, wenn Sie bereit sind.</t>
+  </si>
+  <si>
+    <t>Well done! You have completed the first round. In the next round, you will hear {{num_items}} melodies by two new composers: **{{composer_a}}** and **{{composer_b}}**. Try to figure out which melody belongs to which composer. \\ Press Continue when you are ready.</t>
+  </si>
+  <si>
+    <t>Great work! Now for the final round  featuring {{num_items}} melodies from two more composers: **{{composer_a}}** and **{{composer_b}}**.  \\ Press Continue when you are ready.</t>
+  </si>
+  <si>
+    <t>Super! Jetzt folgt die letzte Runde mit {{num_items}} Melodien von zwei weiteren Komponist*innen: **{{composer_a}}** und **{{composer_b}}**. \\  Drücken Sie Weiter, wenn Sie bereit sind.</t>
+  </si>
+  <si>
+    <t>Super! Jetzt folgt die letzte Runde mit {{num_items}} Melodien von zwei weiteren Komponist*innen: **{{composer_a}}** und **{{composer_b}}**. \\  Drücke Weiter, wenn du bereit bist.</t>
+  </si>
+  <si>
+    <t>In diesem Block hörst du {{num_items}} Melodien von zwei Komponist*innen: **{{composer_a}}** und **{{composer_b}}**. \\ Entscheide intuitiv, wer jede Melodie komponiert hat. Am Anfang wirst du raten müssen. Nutze das Feedback, um dich zu verbessern.</t>
+  </si>
+  <si>
+    <t>In diesem Block hören Sie {{num_items}} Melodien von zwei Komponist*innen: **{{composer_a}}** und **{{composer_b}}**.\\ Entscheiden Sie intuitiv, wer jede Melodie komponiert hat. Am Anfang werden Sie raten müssen.  Nutzen Sie das Feedback, um sich zu verbessern.</t>
+  </si>
+  <si>
+    <t>In this block, you will listen to {{num_items}} melodies by two composers: **{{composer_a}}** and **{{composer_b}}**. \\ Decide intuitively who composed each melody. In the beginning, you will have to guess. Use the feedback to improve over time.</t>
   </si>
 </sst>
 </file>
@@ -920,13 +926,13 @@
         <v>3</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>89</v>
+        <v>120</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>89</v>
+        <v>118</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>88</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="256.5" x14ac:dyDescent="0.45">
@@ -934,13 +940,13 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>106</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
@@ -1074,13 +1080,13 @@
         <v>14</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>90</v>
+        <v>121</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>91</v>
+        <v>122</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>92</v>
+        <v>123</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.45">
@@ -1088,13 +1094,13 @@
         <v>15</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>93</v>
+        <v>124</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>93</v>
+        <v>125</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>93</v>
+        <v>125</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="42.75" x14ac:dyDescent="0.45">
@@ -1158,13 +1164,13 @@
         <v>42</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.45">
@@ -1209,7 +1215,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="114" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:4" ht="128.25" x14ac:dyDescent="0.45">
       <c r="A23" s="1" t="s">
         <v>66</v>
       </c>
@@ -1223,7 +1229,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:4" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A24" s="1" t="s">
         <v>67</v>
       </c>
@@ -1265,107 +1271,107 @@
         <v>74</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:4" ht="57" x14ac:dyDescent="0.45">
       <c r="A27" s="1" t="s">
         <v>76</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>79</v>
+        <v>129</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>80</v>
+        <v>128</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="42.75" x14ac:dyDescent="0.45">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="57" x14ac:dyDescent="0.45">
       <c r="A28" s="1" t="s">
         <v>77</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>82</v>
+        <v>130</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>83</v>
+        <v>131</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="42.75" x14ac:dyDescent="0.45">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="57" x14ac:dyDescent="0.45">
       <c r="A29" s="1" t="s">
         <v>78</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>85</v>
+        <v>132</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>86</v>
+        <v>133</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>87</v>
+        <v>135</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="114" x14ac:dyDescent="0.45">
       <c r="A30" s="1" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>117</v>
+        <v>101</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A31" s="1" t="s">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>119</v>
+        <v>103</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A32" s="1" t="s">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>119</v>
+        <v>103</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A33" s="1" t="s">
-        <v>103</v>
+        <v>88</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A34" s="1" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>71</v>
@@ -1379,91 +1385,91 @@
     </row>
     <row r="35" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A35" s="1" t="s">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>128</v>
+        <v>112</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>129</v>
+        <v>113</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>130</v>
+        <v>114</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A36" s="1" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="B36" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="C36" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A37" s="1" t="s">
-        <v>112</v>
+        <v>96</v>
       </c>
       <c r="B37" t="s">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="C37" t="s">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>114</v>
+        <v>98</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="114" x14ac:dyDescent="0.45">
       <c r="A38" s="1" t="s">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A39" s="1" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>123</v>
+        <v>107</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>123</v>
+        <v>107</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A40" s="1" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>124</v>
+        <v>108</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>124</v>
+        <v>108</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>126</v>
+        <v>110</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A41" s="1" t="s">
-        <v>131</v>
+        <v>115</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>48</v>
@@ -1477,7 +1483,7 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A42" s="1" t="s">
-        <v>132</v>
+        <v>116</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>47</v>
@@ -1486,7 +1492,7 @@
         <v>47</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>133</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changed composer names and demo instruction text
</commit_message>
<xml_diff>
--- a/data_raw/SLT_dict.xlsx
+++ b/data_raw/SLT_dict.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anton\Nextcloud\Promotion\Tests\SLT\data_raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{777569FF-8AEC-4D9E-8A53-B8D2625C002E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{095B305E-678F-4C16-9D60-8EF28DA00716}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="17115" windowHeight="10755" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="149">
   <si>
     <t>key</t>
   </si>
@@ -340,9 +340,6 @@
 Klicken Sie auf die Schaltfläche unten, wenn Sie bereit sind zu beginnen.</t>
   </si>
   <si>
-    <t>On each trial, you will hear a short melody. Your task is to decide which of two composers wrote the melody. Press the corresponding button to give your answer. After each response, you will receive feedback. Click the button below when you are ready to begin.</t>
-  </si>
-  <si>
     <t>Höre dir diese Beispielmelodie an.</t>
   </si>
   <si>
@@ -370,22 +367,10 @@
     <t>COMPOSER_B</t>
   </si>
   <si>
-    <t>Hör dir diese Beispielmelodie an. Wer hat diese Melodie komponiert?</t>
-  </si>
-  <si>
-    <t>Hören Sie sich diese Beispielmelodie an. Wer hat diese Melodie komponiert?</t>
-  </si>
-  <si>
-    <t>Listen to this example melody. Who composed this melody?</t>
-  </si>
-  <si>
     <t>DEMO_CORRECT</t>
   </si>
   <si>
     <t>DEMO_FALSE</t>
-  </si>
-  <si>
-    <t>False.</t>
   </si>
   <si>
     <t>Willkommen zum Statistical Melody Learning Test</t>
@@ -469,6 +454,33 @@
   </si>
   <si>
     <t>In this block, you will listen to {{num_items}} melodies by two composers: **{{composer_a}}** and **{{composer_b}}**. \\ Decide intuitively who composed each melody. In the beginning, you will have to guess. Use the feedback to improve over time.</t>
+  </si>
+  <si>
+    <t>Hören Sie sich diese Beispielmelodie an. Nun müssen Sie *raten*, wer diese Melodie komponiert hat.</t>
+  </si>
+  <si>
+    <t>Listen to this example melody. Now you have to *guess*, who composed this melody.</t>
+  </si>
+  <si>
+    <t>Hör dir diese Beispielmelodie an. Nun musst du *raten*, wer diese Melodie komponiert hat.</t>
+  </si>
+  <si>
+    <t>Du hast richtig geraten!</t>
+  </si>
+  <si>
+    <t>Du hast falsch geraten. Nutze dieses Feedback, um es beim nächsten Versuch besser zu machen.</t>
+  </si>
+  <si>
+    <t>Sie haben richtig geraten!</t>
+  </si>
+  <si>
+    <t>Sie haben falsch geraten. Nutzen Sie dieses Feedback, um es beim nächsten Versuch besser zu machen.</t>
+  </si>
+  <si>
+    <t>Your guess was wrong. Use this feedback for your next trial.</t>
+  </si>
+  <si>
+    <t>On each trial, you will hear a short melody. Your task is to decide which of two composers wrote the melody. Press the corresponding button to give your answer. \\ After each response, you will receive feedback. \\ Click the button below when you are ready to begin.</t>
   </si>
 </sst>
 </file>
@@ -926,13 +938,13 @@
         <v>3</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="256.5" x14ac:dyDescent="0.45">
@@ -946,7 +958,7 @@
         <v>91</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
@@ -1080,13 +1092,13 @@
         <v>14</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.45">
@@ -1094,13 +1106,13 @@
         <v>15</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="42.75" x14ac:dyDescent="0.45">
@@ -1220,13 +1232,13 @@
         <v>66</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="85.5" x14ac:dyDescent="0.45">
@@ -1234,13 +1246,13 @@
         <v>67</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
@@ -1276,13 +1288,13 @@
         <v>76</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="57" x14ac:dyDescent="0.45">
@@ -1290,13 +1302,13 @@
         <v>77</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="57" x14ac:dyDescent="0.45">
@@ -1304,13 +1316,13 @@
         <v>78</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="114" x14ac:dyDescent="0.45">
@@ -1324,7 +1336,7 @@
         <v>101</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>102</v>
+        <v>148</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.45">
@@ -1332,13 +1344,13 @@
         <v>83</v>
       </c>
       <c r="B31" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C31" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="D31" s="2" t="s">
         <v>104</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.45">
@@ -1346,13 +1358,13 @@
         <v>84</v>
       </c>
       <c r="B32" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="D32" s="2" t="s">
         <v>104</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="85.5" x14ac:dyDescent="0.45">
@@ -1383,18 +1395,18 @@
         <v>73</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:4" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A35" s="1" t="s">
         <v>90</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>112</v>
+        <v>142</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>113</v>
+        <v>140</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>114</v>
+        <v>141</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
@@ -1430,69 +1442,69 @@
         <v>99</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A39" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="B39" s="1" t="s">
-        <v>107</v>
-      </c>
       <c r="C39" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A40" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A41" s="1" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>48</v>
+        <v>143</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>48</v>
+        <v>145</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A42" s="1" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>47</v>
+        <v>144</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>47</v>
+        <v>146</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>117</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changed instructions before each block
</commit_message>
<xml_diff>
--- a/data_raw/SLT_dict.xlsx
+++ b/data_raw/SLT_dict.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anton\Nextcloud\Promotion\Tests\SLT\data_raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{095B305E-678F-4C16-9D60-8EF28DA00716}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B811CCB-82E4-4CEF-94C5-417B1E5F7A02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="17115" windowHeight="10755" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -429,33 +429,6 @@
     <t>In the third block, you identified {{number_correct_3}} out of {{total_3}} melodies correctly ({{percent_3}}%).</t>
   </si>
   <si>
-    <t>Gut gemacht! Du hast die erste Runde abgeschlossen. In der nächsten Runde hörst du {{num_items}} Melodien von zwei neuen Komponist*innen: **{{composer_a}}** und **{{composer_b}}**. Versuche herauszufinden, welche Melodie zu wem gehört. \\ Drücke Weiter, wenn du bereit bist.</t>
-  </si>
-  <si>
-    <t>Gut gemacht! Sie haben die erste Runde abgeschlossen. In der nächsten Runde hören Sie {{num_items}} Melodien von zwei neuen Komponist*innen: **{{composer_a}}** und **{{composer_b}}**. Versuche herauszufinden, welche Melodie zu wem gehört. \\ Drücken Sie Weiter, wenn Sie bereit sind.</t>
-  </si>
-  <si>
-    <t>Well done! You have completed the first round. In the next round, you will hear {{num_items}} melodies by two new composers: **{{composer_a}}** and **{{composer_b}}**. Try to figure out which melody belongs to which composer. \\ Press Continue when you are ready.</t>
-  </si>
-  <si>
-    <t>Great work! Now for the final round  featuring {{num_items}} melodies from two more composers: **{{composer_a}}** and **{{composer_b}}**.  \\ Press Continue when you are ready.</t>
-  </si>
-  <si>
-    <t>Super! Jetzt folgt die letzte Runde mit {{num_items}} Melodien von zwei weiteren Komponist*innen: **{{composer_a}}** und **{{composer_b}}**. \\  Drücken Sie Weiter, wenn Sie bereit sind.</t>
-  </si>
-  <si>
-    <t>Super! Jetzt folgt die letzte Runde mit {{num_items}} Melodien von zwei weiteren Komponist*innen: **{{composer_a}}** und **{{composer_b}}**. \\  Drücke Weiter, wenn du bereit bist.</t>
-  </si>
-  <si>
-    <t>In diesem Block hörst du {{num_items}} Melodien von zwei Komponist*innen: **{{composer_a}}** und **{{composer_b}}**. \\ Entscheide intuitiv, wer jede Melodie komponiert hat. Am Anfang wirst du raten müssen. Nutze das Feedback, um dich zu verbessern.</t>
-  </si>
-  <si>
-    <t>In diesem Block hören Sie {{num_items}} Melodien von zwei Komponist*innen: **{{composer_a}}** und **{{composer_b}}**.\\ Entscheiden Sie intuitiv, wer jede Melodie komponiert hat. Am Anfang werden Sie raten müssen.  Nutzen Sie das Feedback, um sich zu verbessern.</t>
-  </si>
-  <si>
-    <t>In this block, you will listen to {{num_items}} melodies by two composers: **{{composer_a}}** and **{{composer_b}}**. \\ Decide intuitively who composed each melody. In the beginning, you will have to guess. Use the feedback to improve over time.</t>
-  </si>
-  <si>
     <t>Hören Sie sich diese Beispielmelodie an. Nun müssen Sie *raten*, wer diese Melodie komponiert hat.</t>
   </si>
   <si>
@@ -481,6 +454,33 @@
   </si>
   <si>
     <t>On each trial, you will hear a short melody. Your task is to decide which of two composers wrote the melody. Press the corresponding button to give your answer. \\ After each response, you will receive feedback. \\ Click the button below when you are ready to begin.</t>
+  </si>
+  <si>
+    <t>In this block, you will listen to {{num_items}} melodies by two composers: **{{composer_a}}** and **{{composer_b}}**. \\ Decide intuitively who composed each melody. In the beginning, you will have to guess, but you can use the feedback to learn and distinguish between the styles of the two composers. Through learning you will improve over time.</t>
+  </si>
+  <si>
+    <t>In diesem Block hören Sie {{num_items}} Melodien von zwei Komponist*innen: **{{composer_a}}** und **{{composer_b}}**.\\ Entscheiden Sie intuitiv, wer jede Melodie komponiert hat. Am Anfang werden Sie raten müssen, aber mit dem Feedback können Sie lernen, die beiden Stile zu unterscheiden. Durch das Lernen werden Sie sich mit der Zeit verbessern.</t>
+  </si>
+  <si>
+    <t>In diesem Block hörst du {{num_items}} Melodien von zwei Komponist*innen: **{{composer_a}}** und **{{composer_b}}**. \\ Entscheide intuitiv, wer jede Melodie komponiert hat. Am Anfang wirst du raten müssen,, aber mit dem Feedback kannst Dulernen, die beiden Stile zu unterscheiden. Durch das Lernen wirst Du dich mit der Zeit verbessern.</t>
+  </si>
+  <si>
+    <t>Gut gemacht! Du hast die erste Runde abgeschlossen. In der nächsten Runde hörst du {{num_items}} Melodien von zwei neuen Komponist*innen: **{{composer_a}}** und **{{composer_b}}**. Versuche zu lernen, welche Melodie zu wem gehört. \\ Drücke Weiter, wenn du bereit bist.</t>
+  </si>
+  <si>
+    <t>Gut gemacht! Sie haben die erste Runde abgeschlossen. In der nächsten Runde hören Sie {{num_items}} Melodien von zwei neuen Komponist*innen: **{{composer_a}}** und **{{composer_b}}**. Versuchen Sie zu lernen, welche Melodie zu wem gehört. \\ Drücken Sie Weiter, wenn Sie bereit sind.</t>
+  </si>
+  <si>
+    <t>Well done! You have completed the first round. In the next round, you will hear {{num_items}} melodies by two new composers: **{{composer_a}}** and **{{composer_b}}**. Try to learn which melody belongs to which composer. \\ Press Continue when you are ready.</t>
+  </si>
+  <si>
+    <t>Great work! Now for the final round  featuring {{num_items}} melodies from two more composers: **{{composer_a}}** and **{{composer_b}}**. \\ Use the feedback to learn to differentiate the melodies.  \\ Press Continue when you are ready.</t>
+  </si>
+  <si>
+    <t>Super! Jetzt folgt die letzte Runde mit {{num_items}} Melodien von zwei weiteren Komponist*innen: **{{composer_a}}** und **{{composer_b}}**. \\ Nutzen Sie das Feedback, um zu lernen die beiden Kompositionsstile zu unterscheiden. \\  Drücken Sie Weiter, wenn Sie bereit sind.</t>
+  </si>
+  <si>
+    <t>Super! Jetzt folgt die letzte Runde mit {{num_items}} Melodien von zwei weiteren Komponist*innen: **{{composer_a}}** und **{{composer_b}}**. \\ Nutze das Feedback, um zu lernen, die beiden Kompositionsstile zu unterscheiden. \\  Drücke Weiter, wenn du bereit bist.</t>
   </si>
 </sst>
 </file>
@@ -591,7 +591,7 @@
         <a:noFill/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
+            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:solidFill>
                 <a:srgbClr val="FFFFFF"/>
               </a:solidFill>
@@ -1232,27 +1232,27 @@
         <v>66</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="85.5" x14ac:dyDescent="0.45">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="114" x14ac:dyDescent="0.45">
       <c r="A24" s="1" t="s">
         <v>67</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
@@ -1336,7 +1336,7 @@
         <v>101</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.45">
@@ -1400,13 +1400,13 @@
         <v>90</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
@@ -1437,18 +1437,18 @@
         <v>98</v>
       </c>
     </row>
-    <row r="38" spans="1:4" ht="114" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:4" ht="156.75" x14ac:dyDescent="0.45">
       <c r="A38" s="1" t="s">
         <v>99</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.45">
@@ -1484,10 +1484,10 @@
         <v>111</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>49</v>
@@ -1498,13 +1498,13 @@
         <v>112</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>

</xml_diff>